<commit_message>
ADX-ddsPIO V2.0 clean up
</commit_message>
<xml_diff>
--- a/doc/ADX-ddsPIO_pinout.xlsx
+++ b/doc/ADX-ddsPIO_pinout.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="10125"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="10201"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/PCOLLA/Documents/GitHub/ADX-ddsPIO/doc/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{19B24FA4-860C-9A4F-9574-DCED952D382D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{528A3C5F-C8DF-4A46-A757-66841E88DAF6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="1320" yWindow="760" windowWidth="26700" windowHeight="16740" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="237" uniqueCount="131">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="239" uniqueCount="131">
   <si>
     <t>Pin</t>
   </si>
@@ -536,7 +536,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="14">
+  <borders count="13">
     <border>
       <left/>
       <right/>
@@ -551,7 +551,7 @@
       <right style="thin">
         <color indexed="64"/>
       </right>
-      <top style="medium">
+      <top style="dotted">
         <color indexed="64"/>
       </top>
       <bottom style="dotted">
@@ -566,7 +566,7 @@
       <right style="thin">
         <color indexed="64"/>
       </right>
-      <top style="medium">
+      <top style="dotted">
         <color indexed="64"/>
       </top>
       <bottom style="dotted">
@@ -581,7 +581,7 @@
       <right style="medium">
         <color indexed="64"/>
       </right>
-      <top style="medium">
+      <top style="dotted">
         <color indexed="64"/>
       </top>
       <bottom style="dotted">
@@ -599,7 +599,7 @@
       <top style="dotted">
         <color indexed="64"/>
       </top>
-      <bottom style="dotted">
+      <bottom style="medium">
         <color indexed="64"/>
       </bottom>
       <diagonal/>
@@ -614,7 +614,7 @@
       <top style="dotted">
         <color indexed="64"/>
       </top>
-      <bottom style="dotted">
+      <bottom style="medium">
         <color indexed="64"/>
       </bottom>
       <diagonal/>
@@ -629,67 +629,9 @@
       <top style="dotted">
         <color indexed="64"/>
       </top>
-      <bottom style="dotted">
+      <bottom style="medium">
         <color indexed="64"/>
       </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="medium">
-        <color indexed="64"/>
-      </left>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top style="dotted">
-        <color indexed="64"/>
-      </top>
-      <bottom style="medium">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top style="dotted">
-        <color indexed="64"/>
-      </top>
-      <bottom style="medium">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right style="medium">
-        <color indexed="64"/>
-      </right>
-      <top style="dotted">
-        <color indexed="64"/>
-      </top>
-      <bottom style="medium">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="medium">
-        <color indexed="64"/>
-      </left>
-      <right style="medium">
-        <color indexed="64"/>
-      </right>
-      <top style="medium">
-        <color indexed="64"/>
-      </top>
-      <bottom/>
       <diagonal/>
     </border>
     <border>
@@ -731,92 +673,128 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="dotted">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="dotted">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="dotted">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="67">
+  <cellXfs count="68">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="5" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="5" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="5" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="5" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="7" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="7" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="7" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="7" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="6" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="6" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="8" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="8" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="7" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="9" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="5" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="11" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="9" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="9" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="9" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="9" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="8" borderId="11" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="7" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="7" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="7" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="6" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="7" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="9" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="7" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="9" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="9" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="9" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="7" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="2" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="3" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="10" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="10" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -825,38 +803,40 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="10" borderId="5" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="10" borderId="6" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="10" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="10" borderId="7" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="10" borderId="8" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
+    <xf numFmtId="0" fontId="2" fillId="10" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="7" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="10" borderId="8" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="10" borderId="9" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="10" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="10" borderId="11" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="10" borderId="12" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="2" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="2" fillId="10" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="10" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="13" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="12" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="12" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="12" borderId="11" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="12" borderId="11" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="11" borderId="11" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="10" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="10" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="9" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="12" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="12" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="12" borderId="7" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="12" borderId="7" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="7" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1140,7 +1120,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="B2:K43"/>
+  <dimension ref="B3:K43"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="3.6640625" customWidth="1"/>
@@ -1149,1097 +1129,1101 @@
     <col min="4" max="5" width="0" hidden="1" customWidth="1"/>
     <col min="6" max="6" width="34.33203125" hidden="1" customWidth="1"/>
     <col min="7" max="7" width="13.1640625" bestFit="1" customWidth="1"/>
-    <col min="8" max="10" width="13.1640625" customWidth="1"/>
+    <col min="8" max="8" width="13.1640625" hidden="1" customWidth="1"/>
+    <col min="9" max="10" width="13.1640625" customWidth="1"/>
     <col min="11" max="11" width="17.6640625" bestFit="1" customWidth="1"/>
     <col min="12" max="12" width="0" hidden="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:11" ht="16" thickBot="1" x14ac:dyDescent="0.25"/>
     <row r="3" spans="2:11" x14ac:dyDescent="0.2">
-      <c r="B3" s="1" t="s">
+      <c r="B3" s="67" t="s">
         <v>0</v>
       </c>
-      <c r="C3" s="2" t="s">
+      <c r="C3" s="67" t="s">
         <v>1</v>
       </c>
-      <c r="D3" s="2" t="s">
+      <c r="D3" s="67" t="s">
         <v>2</v>
       </c>
-      <c r="E3" s="2" t="s">
+      <c r="E3" s="67" t="s">
         <v>3</v>
       </c>
-      <c r="F3" s="3" t="s">
+      <c r="F3" s="67" t="s">
         <v>72</v>
       </c>
-      <c r="G3" s="28" t="s">
+      <c r="G3" s="67" t="s">
         <v>105</v>
       </c>
-      <c r="H3" s="28" t="s">
+      <c r="H3" s="67" t="s">
         <v>126</v>
       </c>
-      <c r="I3" s="28" t="s">
+      <c r="I3" s="67" t="s">
         <v>122</v>
       </c>
-      <c r="J3" s="28" t="s">
+      <c r="J3" s="67" t="s">
         <v>123</v>
       </c>
-      <c r="K3" s="28" t="s">
+      <c r="K3" s="67" t="s">
         <v>107</v>
       </c>
     </row>
     <row r="4" spans="2:11" x14ac:dyDescent="0.2">
-      <c r="B4" s="20">
+      <c r="B4" s="63">
         <f>1</f>
         <v>1</v>
       </c>
-      <c r="C4" s="21" t="s">
+      <c r="C4" s="64" t="s">
         <v>4</v>
       </c>
-      <c r="D4" s="22"/>
-      <c r="E4" s="22" t="s">
+      <c r="D4" s="65"/>
+      <c r="E4" s="65" t="s">
         <v>58</v>
       </c>
-      <c r="F4" s="23" t="s">
+      <c r="F4" s="66" t="s">
         <v>90</v>
       </c>
-      <c r="G4" s="66" t="s">
+      <c r="G4" s="62" t="s">
         <v>106</v>
       </c>
-      <c r="H4" s="66" t="s">
+      <c r="H4" s="62" t="s">
         <v>106</v>
       </c>
-      <c r="I4" s="64" t="s">
+      <c r="I4" s="60" t="s">
         <v>47</v>
       </c>
-      <c r="J4" s="66" t="s">
-        <v>104</v>
-      </c>
-      <c r="K4" s="36"/>
+      <c r="J4" s="62" t="s">
+        <v>104</v>
+      </c>
+      <c r="K4" s="32"/>
     </row>
     <row r="5" spans="2:11" x14ac:dyDescent="0.2">
-      <c r="B5" s="62">
+      <c r="B5" s="58">
         <f>B4+1</f>
         <v>2</v>
       </c>
-      <c r="C5" s="63" t="s">
+      <c r="C5" s="59" t="s">
         <v>5</v>
       </c>
-      <c r="D5" s="22"/>
-      <c r="E5" s="22" t="s">
+      <c r="D5" s="19"/>
+      <c r="E5" s="19" t="s">
         <v>58</v>
       </c>
-      <c r="F5" s="23" t="s">
+      <c r="F5" s="20" t="s">
         <v>90</v>
       </c>
-      <c r="G5" s="64" t="s">
+      <c r="G5" s="60" t="s">
         <v>125</v>
       </c>
-      <c r="H5" s="65" t="s">
+      <c r="H5" s="61" t="s">
         <v>125</v>
       </c>
-      <c r="I5" s="64" t="s">
+      <c r="I5" s="60" t="s">
         <v>48</v>
       </c>
-      <c r="J5" s="65" t="s">
+      <c r="J5" s="61" t="s">
         <v>125</v>
       </c>
-      <c r="K5" s="36"/>
+      <c r="K5" s="32"/>
     </row>
     <row r="6" spans="2:11" x14ac:dyDescent="0.2">
-      <c r="B6" s="8">
+      <c r="B6" s="5">
         <f t="shared" ref="B6:B43" si="0">B5+1</f>
         <v>3</v>
       </c>
-      <c r="C6" s="9" t="s">
+      <c r="C6" s="6" t="s">
         <v>6</v>
       </c>
-      <c r="D6" s="10"/>
-      <c r="E6" s="10"/>
-      <c r="F6" s="11"/>
-      <c r="G6" s="37"/>
-      <c r="H6" s="37"/>
-      <c r="I6" s="37"/>
-      <c r="J6" s="37"/>
-      <c r="K6" s="37"/>
+      <c r="D6" s="7"/>
+      <c r="E6" s="7"/>
+      <c r="F6" s="8"/>
+      <c r="G6" s="33"/>
+      <c r="H6" s="33"/>
+      <c r="I6" s="33"/>
+      <c r="J6" s="33"/>
+      <c r="K6" s="33"/>
     </row>
     <row r="7" spans="2:11" x14ac:dyDescent="0.2">
-      <c r="B7" s="12">
+      <c r="B7" s="9">
         <f t="shared" si="0"/>
         <v>4</v>
       </c>
-      <c r="C7" s="13" t="s">
+      <c r="C7" s="10" t="s">
         <v>7</v>
       </c>
-      <c r="D7" s="14" t="s">
+      <c r="D7" s="11" t="s">
         <v>38</v>
       </c>
-      <c r="E7" s="14" t="s">
+      <c r="E7" s="11" t="s">
         <v>62</v>
       </c>
-      <c r="F7" s="15" t="s">
+      <c r="F7" s="12" t="s">
         <v>69</v>
       </c>
-      <c r="G7" s="29" t="s">
+      <c r="G7" s="25" t="s">
         <v>94</v>
       </c>
-      <c r="H7" s="29" t="s">
+      <c r="H7" s="25" t="s">
         <v>94</v>
       </c>
-      <c r="I7" s="29" t="s">
+      <c r="I7" s="25" t="s">
         <v>94</v>
       </c>
-      <c r="J7" s="29" t="s">
+      <c r="J7" s="25" t="s">
         <v>94</v>
       </c>
-      <c r="K7" s="29" t="s">
+      <c r="K7" s="25" t="s">
         <v>95</v>
       </c>
     </row>
     <row r="8" spans="2:11" x14ac:dyDescent="0.2">
-      <c r="B8" s="12">
+      <c r="B8" s="9">
         <f t="shared" si="0"/>
         <v>5</v>
       </c>
-      <c r="C8" s="13" t="s">
+      <c r="C8" s="10" t="s">
         <v>8</v>
       </c>
-      <c r="D8" s="14" t="s">
+      <c r="D8" s="11" t="s">
         <v>39</v>
       </c>
-      <c r="E8" s="14" t="s">
+      <c r="E8" s="11" t="s">
         <v>63</v>
       </c>
-      <c r="F8" s="15" t="s">
+      <c r="F8" s="12" t="s">
         <v>69</v>
       </c>
-      <c r="G8" s="29" t="s">
+      <c r="G8" s="25" t="s">
         <v>75</v>
       </c>
-      <c r="H8" s="29" t="s">
+      <c r="H8" s="25" t="s">
         <v>75</v>
       </c>
-      <c r="I8" s="29" t="s">
+      <c r="I8" s="25" t="s">
         <v>75</v>
       </c>
-      <c r="J8" s="29" t="s">
+      <c r="J8" s="25" t="s">
         <v>75</v>
       </c>
-      <c r="K8" s="29" t="s">
+      <c r="K8" s="25" t="s">
         <v>96</v>
       </c>
     </row>
     <row r="9" spans="2:11" x14ac:dyDescent="0.2">
-      <c r="B9" s="12">
+      <c r="B9" s="9">
         <f t="shared" si="0"/>
         <v>6</v>
       </c>
-      <c r="C9" s="13" t="s">
+      <c r="C9" s="10" t="s">
         <v>9</v>
       </c>
-      <c r="D9" s="14" t="s">
+      <c r="D9" s="11" t="s">
         <v>40</v>
       </c>
-      <c r="E9" s="14" t="s">
+      <c r="E9" s="11" t="s">
         <v>64</v>
       </c>
-      <c r="F9" s="15" t="s">
+      <c r="F9" s="12" t="s">
         <v>69</v>
       </c>
-      <c r="G9" s="29" t="s">
+      <c r="G9" s="25" t="s">
         <v>73</v>
       </c>
-      <c r="H9" s="29" t="s">
+      <c r="H9" s="25" t="s">
         <v>73</v>
       </c>
-      <c r="I9" s="29" t="s">
+      <c r="I9" s="25" t="s">
         <v>73</v>
       </c>
-      <c r="J9" s="29" t="s">
+      <c r="J9" s="25" t="s">
         <v>73</v>
       </c>
-      <c r="K9" s="29" t="s">
+      <c r="K9" s="25" t="s">
         <v>97</v>
       </c>
     </row>
     <row r="10" spans="2:11" x14ac:dyDescent="0.2">
-      <c r="B10" s="12">
+      <c r="B10" s="9">
         <f t="shared" si="0"/>
         <v>7</v>
       </c>
-      <c r="C10" s="13" t="s">
+      <c r="C10" s="10" t="s">
         <v>10</v>
       </c>
-      <c r="D10" s="14" t="s">
+      <c r="D10" s="11" t="s">
         <v>41</v>
       </c>
-      <c r="E10" s="14" t="s">
+      <c r="E10" s="11" t="s">
         <v>65</v>
       </c>
-      <c r="F10" s="15" t="s">
+      <c r="F10" s="12" t="s">
         <v>69</v>
       </c>
-      <c r="G10" s="29" t="s">
+      <c r="G10" s="25" t="s">
         <v>74</v>
       </c>
-      <c r="H10" s="29" t="s">
+      <c r="H10" s="25" t="s">
         <v>74</v>
       </c>
-      <c r="I10" s="29" t="s">
+      <c r="I10" s="25" t="s">
         <v>74</v>
       </c>
-      <c r="J10" s="29" t="s">
+      <c r="J10" s="25" t="s">
         <v>74</v>
       </c>
-      <c r="K10" s="29" t="s">
+      <c r="K10" s="25" t="s">
         <v>98</v>
       </c>
     </row>
     <row r="11" spans="2:11" x14ac:dyDescent="0.2">
-      <c r="B11" s="8">
+      <c r="B11" s="5">
         <f t="shared" si="0"/>
         <v>8</v>
       </c>
-      <c r="C11" s="9" t="s">
+      <c r="C11" s="6" t="s">
         <v>6</v>
       </c>
-      <c r="D11" s="10"/>
-      <c r="E11" s="10"/>
-      <c r="F11" s="11"/>
-      <c r="G11" s="37"/>
-      <c r="H11" s="37"/>
-      <c r="I11" s="37"/>
-      <c r="J11" s="37"/>
-      <c r="K11" s="37"/>
+      <c r="D11" s="7"/>
+      <c r="E11" s="7"/>
+      <c r="F11" s="8"/>
+      <c r="G11" s="33"/>
+      <c r="H11" s="33"/>
+      <c r="I11" s="33"/>
+      <c r="J11" s="33"/>
+      <c r="K11" s="33"/>
     </row>
     <row r="12" spans="2:11" x14ac:dyDescent="0.2">
-      <c r="B12" s="12">
+      <c r="B12" s="9">
         <f t="shared" si="0"/>
         <v>9</v>
       </c>
-      <c r="C12" s="13" t="s">
+      <c r="C12" s="10" t="s">
         <v>11</v>
       </c>
-      <c r="D12" s="6" t="s">
+      <c r="D12" s="3" t="s">
         <v>42</v>
       </c>
-      <c r="E12" s="6" t="s">
+      <c r="E12" s="3" t="s">
         <v>66</v>
       </c>
-      <c r="F12" s="7" t="s">
+      <c r="F12" s="4" t="s">
         <v>69</v>
       </c>
-      <c r="G12" s="43" t="s">
+      <c r="G12" s="39" t="s">
         <v>112</v>
       </c>
-      <c r="H12" s="43" t="s">
+      <c r="H12" s="39" t="s">
         <v>112</v>
       </c>
-      <c r="I12" s="43" t="s">
+      <c r="I12" s="39" t="s">
         <v>112</v>
       </c>
-      <c r="J12" s="43" t="s">
+      <c r="J12" s="39" t="s">
         <v>112</v>
       </c>
-      <c r="K12" s="29" t="s">
+      <c r="K12" s="25" t="s">
         <v>109</v>
       </c>
     </row>
     <row r="13" spans="2:11" x14ac:dyDescent="0.2">
-      <c r="B13" s="12">
+      <c r="B13" s="9">
         <f t="shared" si="0"/>
         <v>10</v>
       </c>
-      <c r="C13" s="13" t="s">
+      <c r="C13" s="10" t="s">
         <v>12</v>
       </c>
-      <c r="D13" s="14" t="s">
+      <c r="D13" s="11" t="s">
         <v>43</v>
       </c>
-      <c r="E13" s="14" t="s">
+      <c r="E13" s="11" t="s">
         <v>67</v>
       </c>
-      <c r="F13" s="15" t="s">
+      <c r="F13" s="12" t="s">
         <v>69</v>
       </c>
-      <c r="G13" s="43" t="s">
+      <c r="G13" s="39" t="s">
         <v>113</v>
       </c>
-      <c r="H13" s="43" t="s">
+      <c r="H13" s="39" t="s">
         <v>113</v>
       </c>
-      <c r="I13" s="43" t="s">
+      <c r="I13" s="39" t="s">
         <v>113</v>
       </c>
-      <c r="J13" s="43" t="s">
+      <c r="J13" s="39" t="s">
         <v>113</v>
       </c>
-      <c r="K13" s="43" t="s">
+      <c r="K13" s="39" t="s">
         <v>116</v>
       </c>
     </row>
     <row r="14" spans="2:11" x14ac:dyDescent="0.2">
-      <c r="B14" s="38">
+      <c r="B14" s="34">
         <f t="shared" si="0"/>
         <v>11</v>
       </c>
-      <c r="C14" s="39" t="s">
+      <c r="C14" s="35" t="s">
         <v>13</v>
       </c>
-      <c r="D14" s="14" t="s">
+      <c r="D14" s="11" t="s">
         <v>44</v>
       </c>
-      <c r="E14" s="14" t="s">
+      <c r="E14" s="11" t="s">
         <v>68</v>
       </c>
-      <c r="F14" s="15" t="s">
+      <c r="F14" s="12" t="s">
         <v>88</v>
       </c>
-      <c r="G14" s="44" t="s">
+      <c r="G14" s="40" t="s">
         <v>114</v>
       </c>
-      <c r="H14" s="44" t="s">
+      <c r="H14" s="40" t="s">
         <v>114</v>
       </c>
-      <c r="I14" s="44" t="s">
+      <c r="I14" s="40" t="s">
         <v>114</v>
       </c>
-      <c r="J14" s="44" t="s">
+      <c r="J14" s="40" t="s">
         <v>114</v>
       </c>
-      <c r="K14" s="44" t="s">
+      <c r="K14" s="40" t="s">
         <v>115</v>
       </c>
     </row>
     <row r="15" spans="2:11" x14ac:dyDescent="0.2">
-      <c r="B15" s="62">
+      <c r="B15" s="58">
         <f t="shared" si="0"/>
         <v>12</v>
       </c>
-      <c r="C15" s="63" t="s">
+      <c r="C15" s="59" t="s">
         <v>14</v>
       </c>
-      <c r="D15" s="16"/>
-      <c r="E15" s="16" t="s">
+      <c r="D15" s="13"/>
+      <c r="E15" s="13" t="s">
         <v>59</v>
       </c>
-      <c r="F15" s="17" t="s">
+      <c r="F15" s="14" t="s">
         <v>89</v>
       </c>
-      <c r="G15" s="43" t="s">
+      <c r="G15" s="39" t="s">
         <v>118</v>
       </c>
-      <c r="H15" s="43" t="s">
+      <c r="H15" s="39" t="s">
         <v>118</v>
       </c>
-      <c r="I15" s="64" t="s">
+      <c r="I15" s="60" t="s">
         <v>125</v>
       </c>
-      <c r="J15" s="43" t="s">
+      <c r="J15" s="39" t="s">
         <v>118</v>
       </c>
-      <c r="K15" s="29" t="s">
+      <c r="K15" s="25" t="s">
         <v>119</v>
       </c>
     </row>
     <row r="16" spans="2:11" x14ac:dyDescent="0.2">
-      <c r="B16" s="8">
+      <c r="B16" s="5">
         <f t="shared" si="0"/>
         <v>13</v>
       </c>
-      <c r="C16" s="9" t="s">
+      <c r="C16" s="6" t="s">
         <v>6</v>
       </c>
-      <c r="D16" s="10"/>
-      <c r="E16" s="10"/>
-      <c r="F16" s="11"/>
-      <c r="G16" s="37"/>
-      <c r="H16" s="37"/>
-      <c r="I16" s="37"/>
-      <c r="J16" s="37"/>
-      <c r="K16" s="37"/>
+      <c r="D16" s="7"/>
+      <c r="E16" s="7"/>
+      <c r="F16" s="8"/>
+      <c r="G16" s="33"/>
+      <c r="H16" s="33"/>
+      <c r="I16" s="33"/>
+      <c r="J16" s="33"/>
+      <c r="K16" s="33"/>
     </row>
     <row r="17" spans="2:11" x14ac:dyDescent="0.2">
-      <c r="B17" s="38">
+      <c r="B17" s="34">
         <f t="shared" si="0"/>
         <v>14</v>
       </c>
-      <c r="C17" s="39" t="s">
+      <c r="C17" s="35" t="s">
         <v>15</v>
       </c>
-      <c r="D17" s="6"/>
-      <c r="E17" s="6" t="s">
+      <c r="D17" s="3"/>
+      <c r="E17" s="3" t="s">
         <v>58</v>
       </c>
-      <c r="F17" s="7" t="s">
+      <c r="F17" s="4" t="s">
         <v>80</v>
       </c>
-      <c r="G17" s="44" t="s">
+      <c r="G17" s="40" t="s">
         <v>91</v>
       </c>
-      <c r="H17" s="44" t="s">
+      <c r="H17" s="40" t="s">
         <v>91</v>
       </c>
-      <c r="I17" s="44" t="s">
+      <c r="I17" s="40" t="s">
         <v>91</v>
       </c>
-      <c r="J17" s="44" t="s">
+      <c r="J17" s="40" t="s">
         <v>91</v>
       </c>
-      <c r="K17" s="30" t="s">
+      <c r="K17" s="26" t="s">
         <v>110</v>
       </c>
     </row>
     <row r="18" spans="2:11" x14ac:dyDescent="0.2">
-      <c r="B18" s="38">
+      <c r="B18" s="34">
         <f t="shared" si="0"/>
         <v>15</v>
       </c>
-      <c r="C18" s="39" t="s">
+      <c r="C18" s="35" t="s">
         <v>16</v>
       </c>
-      <c r="D18" s="6"/>
-      <c r="E18" s="6" t="s">
+      <c r="D18" s="3"/>
+      <c r="E18" s="3" t="s">
         <v>58</v>
       </c>
-      <c r="F18" s="7" t="s">
+      <c r="F18" s="4" t="s">
         <v>81</v>
       </c>
-      <c r="G18" s="44" t="s">
+      <c r="G18" s="40" t="s">
         <v>92</v>
       </c>
-      <c r="H18" s="44" t="s">
+      <c r="H18" s="40" t="s">
         <v>92</v>
       </c>
-      <c r="I18" s="44" t="s">
+      <c r="I18" s="40" t="s">
         <v>92</v>
       </c>
-      <c r="J18" s="44" t="s">
+      <c r="J18" s="40" t="s">
         <v>92</v>
       </c>
-      <c r="K18" s="30" t="s">
+      <c r="K18" s="26" t="s">
         <v>111</v>
       </c>
     </row>
     <row r="19" spans="2:11" x14ac:dyDescent="0.2">
-      <c r="B19" s="4">
+      <c r="B19" s="1">
         <f t="shared" si="0"/>
         <v>16</v>
       </c>
-      <c r="C19" s="5" t="s">
+      <c r="C19" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="D19" s="40" t="s">
+      <c r="D19" s="36" t="s">
         <v>45</v>
       </c>
-      <c r="E19" s="40" t="s">
+      <c r="E19" s="36" t="s">
         <v>61</v>
       </c>
-      <c r="F19" s="41" t="s">
+      <c r="F19" s="37" t="s">
         <v>78</v>
       </c>
-      <c r="G19" s="58" t="s">
+      <c r="G19" s="54" t="s">
         <v>120</v>
       </c>
-      <c r="H19" s="58" t="s">
+      <c r="H19" s="54" t="s">
         <v>120</v>
       </c>
-      <c r="I19" s="58" t="s">
+      <c r="I19" s="54" t="s">
         <v>120</v>
       </c>
-      <c r="J19" s="58" t="s">
+      <c r="J19" s="54" t="s">
         <v>120</v>
       </c>
-      <c r="K19" s="32" t="s">
+      <c r="K19" s="28" t="s">
         <v>121</v>
       </c>
     </row>
     <row r="20" spans="2:11" x14ac:dyDescent="0.2">
-      <c r="B20" s="4">
+      <c r="B20" s="1">
         <f t="shared" si="0"/>
         <v>17</v>
       </c>
-      <c r="C20" s="5" t="s">
+      <c r="C20" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="D20" s="6" t="s">
+      <c r="D20" s="3" t="s">
         <v>45</v>
       </c>
-      <c r="E20" s="6" t="s">
+      <c r="E20" s="3" t="s">
         <v>60</v>
       </c>
-      <c r="F20" s="7" t="s">
+      <c r="F20" s="4" t="s">
         <v>79</v>
       </c>
-      <c r="G20" s="32" t="s">
+      <c r="G20" s="28" t="s">
         <v>108</v>
       </c>
-      <c r="H20" s="32" t="s">
+      <c r="H20" s="28" t="s">
         <v>108</v>
       </c>
-      <c r="I20" s="32" t="s">
+      <c r="I20" s="28" t="s">
         <v>108</v>
       </c>
-      <c r="J20" s="32" t="s">
+      <c r="J20" s="28" t="s">
         <v>108</v>
       </c>
-      <c r="K20" s="32" t="s">
+      <c r="K20" s="28" t="s">
         <v>117</v>
       </c>
     </row>
     <row r="21" spans="2:11" x14ac:dyDescent="0.2">
-      <c r="B21" s="8">
+      <c r="B21" s="5">
         <f t="shared" si="0"/>
         <v>18</v>
       </c>
-      <c r="C21" s="9" t="s">
+      <c r="C21" s="6" t="s">
         <v>6</v>
       </c>
-      <c r="D21" s="10"/>
-      <c r="E21" s="10"/>
-      <c r="F21" s="11"/>
-      <c r="G21" s="37"/>
-      <c r="H21" s="37"/>
-      <c r="I21" s="37"/>
-      <c r="J21" s="37"/>
-      <c r="K21" s="37"/>
+      <c r="D21" s="7"/>
+      <c r="E21" s="7"/>
+      <c r="F21" s="8"/>
+      <c r="G21" s="33"/>
+      <c r="H21" s="33"/>
+      <c r="I21" s="33"/>
+      <c r="J21" s="33"/>
+      <c r="K21" s="33"/>
     </row>
     <row r="22" spans="2:11" x14ac:dyDescent="0.2">
-      <c r="B22" s="4">
+      <c r="B22" s="1">
         <f t="shared" si="0"/>
         <v>19</v>
       </c>
-      <c r="C22" s="5" t="s">
+      <c r="C22" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="D22" s="6"/>
-      <c r="E22" s="6" t="s">
+      <c r="D22" s="3"/>
+      <c r="E22" s="3" t="s">
         <v>56</v>
       </c>
-      <c r="F22" s="7" t="s">
+      <c r="F22" s="4" t="s">
         <v>82</v>
       </c>
-      <c r="G22" s="32" t="s">
+      <c r="G22" s="28" t="s">
         <v>127</v>
       </c>
-      <c r="H22" s="32" t="s">
+      <c r="H22" s="28" t="s">
         <v>128</v>
       </c>
-      <c r="I22" s="32" t="s">
+      <c r="I22" s="28" t="s">
         <v>127</v>
       </c>
-      <c r="J22" s="32" t="s">
+      <c r="J22" s="28" t="s">
         <v>127</v>
       </c>
-      <c r="K22" s="32" t="s">
+      <c r="K22" s="28" t="s">
         <v>129</v>
       </c>
     </row>
     <row r="23" spans="2:11" x14ac:dyDescent="0.2">
-      <c r="B23" s="4">
+      <c r="B23" s="1">
         <f t="shared" si="0"/>
         <v>20</v>
       </c>
-      <c r="C23" s="5" t="s">
+      <c r="C23" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="D23" s="6"/>
-      <c r="E23" s="6" t="s">
+      <c r="D23" s="3"/>
+      <c r="E23" s="3" t="s">
         <v>46</v>
       </c>
-      <c r="F23" s="7" t="s">
+      <c r="F23" s="4" t="s">
         <v>77</v>
       </c>
-      <c r="G23" s="32" t="s">
+      <c r="G23" s="28" t="s">
         <v>124</v>
       </c>
-      <c r="H23" s="32" t="s">
+      <c r="H23" s="28" t="s">
         <v>124</v>
       </c>
-      <c r="I23" s="32" t="s">
+      <c r="I23" s="28" t="s">
         <v>124</v>
       </c>
-      <c r="J23" s="32" t="s">
+      <c r="J23" s="28" t="s">
         <v>124</v>
       </c>
-      <c r="K23" s="32" t="s">
+      <c r="K23" s="28" t="s">
         <v>124</v>
       </c>
     </row>
     <row r="24" spans="2:11" x14ac:dyDescent="0.2">
-      <c r="B24" s="62">
+      <c r="B24" s="58">
         <f t="shared" si="0"/>
         <v>21</v>
       </c>
-      <c r="C24" s="63" t="s">
+      <c r="C24" s="59" t="s">
         <v>21</v>
       </c>
-      <c r="D24" s="33"/>
-      <c r="E24" s="33" t="s">
+      <c r="D24" s="29"/>
+      <c r="E24" s="29" t="s">
         <v>47</v>
       </c>
-      <c r="F24" s="34" t="s">
+      <c r="F24" s="30" t="s">
         <v>70</v>
       </c>
-      <c r="G24" s="66" t="s">
-        <v>104</v>
-      </c>
-      <c r="H24" s="66" t="s">
-        <v>104</v>
-      </c>
-      <c r="I24" s="61"/>
-      <c r="J24" s="64" t="s">
+      <c r="G24" s="60" t="s">
         <v>47</v>
       </c>
-      <c r="K24" s="66"/>
+      <c r="H24" s="60" t="s">
+        <v>47</v>
+      </c>
+      <c r="I24" s="57"/>
+      <c r="J24" s="60" t="s">
+        <v>47</v>
+      </c>
+      <c r="K24" s="62"/>
     </row>
     <row r="25" spans="2:11" x14ac:dyDescent="0.2">
-      <c r="B25" s="62">
+      <c r="B25" s="58">
         <f t="shared" si="0"/>
         <v>22</v>
       </c>
-      <c r="C25" s="63" t="s">
+      <c r="C25" s="59" t="s">
         <v>22</v>
       </c>
-      <c r="D25" s="33"/>
-      <c r="E25" s="33" t="s">
+      <c r="D25" s="29"/>
+      <c r="E25" s="29" t="s">
         <v>48</v>
       </c>
-      <c r="F25" s="34" t="s">
+      <c r="F25" s="30" t="s">
         <v>70</v>
       </c>
-      <c r="G25" s="66" t="s">
-        <v>104</v>
-      </c>
-      <c r="H25" s="66" t="s">
-        <v>104</v>
-      </c>
-      <c r="I25" s="61"/>
-      <c r="J25" s="64" t="s">
+      <c r="G25" s="60" t="s">
         <v>48</v>
       </c>
-      <c r="K25" s="66"/>
+      <c r="H25" s="60" t="s">
+        <v>48</v>
+      </c>
+      <c r="I25" s="57"/>
+      <c r="J25" s="60" t="s">
+        <v>48</v>
+      </c>
+      <c r="K25" s="62"/>
     </row>
     <row r="26" spans="2:11" x14ac:dyDescent="0.2">
-      <c r="B26" s="8">
+      <c r="B26" s="5">
         <f t="shared" si="0"/>
         <v>23</v>
       </c>
-      <c r="C26" s="9" t="s">
+      <c r="C26" s="6" t="s">
         <v>6</v>
       </c>
-      <c r="D26" s="10"/>
-      <c r="E26" s="10"/>
-      <c r="F26" s="11"/>
-      <c r="G26" s="37"/>
-      <c r="H26" s="37"/>
-      <c r="I26" s="61"/>
-      <c r="J26" s="37"/>
-      <c r="K26" s="37"/>
+      <c r="D26" s="7"/>
+      <c r="E26" s="7"/>
+      <c r="F26" s="8"/>
+      <c r="G26" s="33"/>
+      <c r="H26" s="33"/>
+      <c r="I26" s="57"/>
+      <c r="J26" s="33"/>
+      <c r="K26" s="33"/>
     </row>
     <row r="27" spans="2:11" x14ac:dyDescent="0.2">
-      <c r="B27" s="20">
+      <c r="B27" s="17">
         <f t="shared" si="0"/>
         <v>24</v>
       </c>
-      <c r="C27" s="21" t="s">
+      <c r="C27" s="18" t="s">
         <v>23</v>
       </c>
-      <c r="D27" s="22"/>
-      <c r="E27" s="22" t="s">
+      <c r="D27" s="19"/>
+      <c r="E27" s="19" t="s">
         <v>49</v>
       </c>
-      <c r="F27" s="23" t="s">
+      <c r="F27" s="20" t="s">
         <v>83</v>
       </c>
-      <c r="G27" s="66" t="s">
-        <v>104</v>
-      </c>
-      <c r="H27" s="66" t="s">
-        <v>104</v>
-      </c>
-      <c r="I27" s="61"/>
-      <c r="J27" s="66" t="s">
-        <v>104</v>
-      </c>
-      <c r="K27" s="66"/>
+      <c r="G27" s="62" t="s">
+        <v>104</v>
+      </c>
+      <c r="H27" s="62" t="s">
+        <v>104</v>
+      </c>
+      <c r="I27" s="57"/>
+      <c r="J27" s="62" t="s">
+        <v>104</v>
+      </c>
+      <c r="K27" s="62"/>
     </row>
     <row r="28" spans="2:11" x14ac:dyDescent="0.2">
-      <c r="B28" s="20">
+      <c r="B28" s="17">
         <f t="shared" si="0"/>
         <v>25</v>
       </c>
-      <c r="C28" s="21" t="s">
+      <c r="C28" s="18" t="s">
         <v>24</v>
       </c>
-      <c r="D28" s="22" t="s">
+      <c r="D28" s="19" t="s">
         <v>50</v>
       </c>
-      <c r="E28" s="22" t="s">
+      <c r="E28" s="19" t="s">
         <v>53</v>
       </c>
-      <c r="F28" s="23" t="s">
+      <c r="F28" s="20" t="s">
         <v>84</v>
       </c>
-      <c r="G28" s="66" t="s">
-        <v>104</v>
-      </c>
-      <c r="H28" s="66" t="s">
-        <v>104</v>
-      </c>
-      <c r="I28" s="61"/>
-      <c r="J28" s="66" t="s">
-        <v>104</v>
-      </c>
-      <c r="K28" s="66"/>
+      <c r="G28" s="62" t="s">
+        <v>104</v>
+      </c>
+      <c r="H28" s="62" t="s">
+        <v>104</v>
+      </c>
+      <c r="I28" s="57"/>
+      <c r="J28" s="62" t="s">
+        <v>104</v>
+      </c>
+      <c r="K28" s="62"/>
     </row>
     <row r="29" spans="2:11" x14ac:dyDescent="0.2">
-      <c r="B29" s="20">
+      <c r="B29" s="17">
         <f t="shared" si="0"/>
         <v>26</v>
       </c>
-      <c r="C29" s="21" t="s">
+      <c r="C29" s="18" t="s">
         <v>25</v>
       </c>
-      <c r="D29" s="22" t="s">
+      <c r="D29" s="19" t="s">
         <v>50</v>
       </c>
-      <c r="E29" s="22" t="s">
+      <c r="E29" s="19" t="s">
         <v>54</v>
       </c>
-      <c r="F29" s="23" t="s">
+      <c r="F29" s="20" t="s">
         <v>85</v>
       </c>
-      <c r="G29" s="66" t="s">
-        <v>104</v>
-      </c>
-      <c r="H29" s="66" t="s">
-        <v>104</v>
-      </c>
-      <c r="I29" s="61"/>
-      <c r="J29" s="66" t="s">
-        <v>104</v>
-      </c>
-      <c r="K29" s="66"/>
+      <c r="G29" s="62" t="s">
+        <v>104</v>
+      </c>
+      <c r="H29" s="62" t="s">
+        <v>104</v>
+      </c>
+      <c r="I29" s="57"/>
+      <c r="J29" s="62" t="s">
+        <v>104</v>
+      </c>
+      <c r="K29" s="62"/>
     </row>
     <row r="30" spans="2:11" x14ac:dyDescent="0.2">
-      <c r="B30" s="20">
+      <c r="B30" s="17">
         <f t="shared" si="0"/>
         <v>27</v>
       </c>
-      <c r="C30" s="21" t="s">
+      <c r="C30" s="18" t="s">
         <v>26</v>
       </c>
-      <c r="D30" s="22" t="s">
+      <c r="D30" s="19" t="s">
         <v>50</v>
       </c>
-      <c r="E30" s="22" t="s">
+      <c r="E30" s="19" t="s">
         <v>55</v>
       </c>
-      <c r="F30" s="23" t="s">
+      <c r="F30" s="20" t="s">
         <v>86</v>
       </c>
-      <c r="G30" s="66" t="s">
-        <v>104</v>
-      </c>
-      <c r="H30" s="66" t="s">
-        <v>104</v>
-      </c>
-      <c r="I30" s="61"/>
-      <c r="J30" s="66" t="s">
-        <v>104</v>
-      </c>
-      <c r="K30" s="66"/>
+      <c r="G30" s="62" t="s">
+        <v>104</v>
+      </c>
+      <c r="H30" s="62" t="s">
+        <v>104</v>
+      </c>
+      <c r="I30" s="57"/>
+      <c r="J30" s="62" t="s">
+        <v>104</v>
+      </c>
+      <c r="K30" s="62"/>
     </row>
     <row r="31" spans="2:11" x14ac:dyDescent="0.2">
-      <c r="B31" s="8">
+      <c r="B31" s="5">
         <f t="shared" si="0"/>
         <v>28</v>
       </c>
-      <c r="C31" s="9" t="s">
+      <c r="C31" s="6" t="s">
         <v>6</v>
       </c>
-      <c r="D31" s="10"/>
-      <c r="E31" s="10"/>
-      <c r="F31" s="11"/>
-      <c r="G31" s="37"/>
-      <c r="H31" s="37"/>
-      <c r="I31" s="61"/>
-      <c r="J31" s="37"/>
-      <c r="K31" s="37"/>
+      <c r="D31" s="7"/>
+      <c r="E31" s="7"/>
+      <c r="F31" s="8"/>
+      <c r="G31" s="33"/>
+      <c r="H31" s="33"/>
+      <c r="I31" s="57"/>
+      <c r="J31" s="33"/>
+      <c r="K31" s="33"/>
     </row>
     <row r="32" spans="2:11" x14ac:dyDescent="0.2">
-      <c r="B32" s="20">
+      <c r="B32" s="17">
         <f t="shared" si="0"/>
         <v>29</v>
       </c>
-      <c r="C32" s="21" t="s">
+      <c r="C32" s="18" t="s">
         <v>27</v>
       </c>
-      <c r="D32" s="22"/>
-      <c r="E32" s="22" t="s">
+      <c r="D32" s="19"/>
+      <c r="E32" s="19" t="s">
         <v>57</v>
       </c>
-      <c r="F32" s="23" t="s">
+      <c r="F32" s="20" t="s">
         <v>87</v>
       </c>
-      <c r="G32" s="66" t="s">
-        <v>104</v>
-      </c>
-      <c r="H32" s="66" t="s">
-        <v>104</v>
-      </c>
-      <c r="I32" s="61"/>
-      <c r="J32" s="66" t="s">
-        <v>104</v>
-      </c>
-      <c r="K32" s="66"/>
+      <c r="G32" s="62" t="s">
+        <v>104</v>
+      </c>
+      <c r="H32" s="62" t="s">
+        <v>104</v>
+      </c>
+      <c r="I32" s="57"/>
+      <c r="J32" s="62" t="s">
+        <v>104</v>
+      </c>
+      <c r="K32" s="62"/>
     </row>
     <row r="33" spans="2:11" x14ac:dyDescent="0.2">
-      <c r="B33" s="20">
+      <c r="B33" s="17">
         <f t="shared" si="0"/>
         <v>30</v>
       </c>
-      <c r="C33" s="21" t="s">
+      <c r="C33" s="18" t="s">
         <v>28</v>
       </c>
-      <c r="D33" s="22"/>
-      <c r="E33" s="22"/>
-      <c r="F33" s="23"/>
-      <c r="G33" s="66" t="s">
-        <v>104</v>
-      </c>
-      <c r="H33" s="66" t="s">
-        <v>104</v>
-      </c>
-      <c r="I33" s="61"/>
-      <c r="J33" s="66" t="s">
-        <v>104</v>
-      </c>
-      <c r="K33" s="66"/>
+      <c r="D33" s="19"/>
+      <c r="E33" s="19"/>
+      <c r="F33" s="20"/>
+      <c r="G33" s="62" t="s">
+        <v>104</v>
+      </c>
+      <c r="H33" s="62" t="s">
+        <v>104</v>
+      </c>
+      <c r="I33" s="57"/>
+      <c r="J33" s="62" t="s">
+        <v>104</v>
+      </c>
+      <c r="K33" s="62"/>
     </row>
     <row r="34" spans="2:11" x14ac:dyDescent="0.2">
-      <c r="B34" s="18">
+      <c r="B34" s="15">
         <f t="shared" si="0"/>
         <v>31</v>
       </c>
-      <c r="C34" s="19" t="s">
+      <c r="C34" s="16" t="s">
         <v>29</v>
       </c>
-      <c r="D34" s="22"/>
-      <c r="E34" s="22" t="s">
+      <c r="D34" s="19"/>
+      <c r="E34" s="19" t="s">
         <v>51</v>
       </c>
-      <c r="F34" s="23" t="s">
+      <c r="F34" s="20" t="s">
         <v>71</v>
       </c>
-      <c r="G34" s="66" t="s">
-        <v>104</v>
-      </c>
-      <c r="H34" s="42" t="s">
+      <c r="G34" s="38" t="s">
         <v>118</v>
       </c>
-      <c r="I34" s="42" t="s">
+      <c r="H34" s="38" t="s">
         <v>118</v>
       </c>
-      <c r="J34" s="42" t="s">
+      <c r="I34" s="38" t="s">
         <v>118</v>
       </c>
-      <c r="K34" s="42" t="s">
+      <c r="J34" s="38" t="s">
+        <v>118</v>
+      </c>
+      <c r="K34" s="38" t="s">
         <v>130</v>
       </c>
     </row>
     <row r="35" spans="2:11" x14ac:dyDescent="0.2">
-      <c r="B35" s="20">
+      <c r="B35" s="17">
         <f t="shared" si="0"/>
         <v>32</v>
       </c>
-      <c r="C35" s="21" t="s">
+      <c r="C35" s="18" t="s">
         <v>30</v>
       </c>
-      <c r="D35" s="22"/>
-      <c r="E35" s="22" t="s">
+      <c r="D35" s="19"/>
+      <c r="E35" s="19" t="s">
         <v>52</v>
       </c>
-      <c r="F35" s="23" t="s">
+      <c r="F35" s="20" t="s">
         <v>76</v>
       </c>
-      <c r="G35" s="66" t="s">
-        <v>104</v>
-      </c>
-      <c r="H35" s="66" t="s">
-        <v>104</v>
-      </c>
-      <c r="I35" s="66" t="s">
-        <v>104</v>
-      </c>
-      <c r="J35" s="66" t="s">
-        <v>104</v>
-      </c>
-      <c r="K35" s="66" t="s">
+      <c r="G35" s="62" t="s">
+        <v>104</v>
+      </c>
+      <c r="H35" s="62" t="s">
+        <v>104</v>
+      </c>
+      <c r="I35" s="62" t="s">
+        <v>104</v>
+      </c>
+      <c r="J35" s="62" t="s">
+        <v>104</v>
+      </c>
+      <c r="K35" s="62" t="s">
         <v>104</v>
       </c>
     </row>
     <row r="36" spans="2:11" x14ac:dyDescent="0.2">
-      <c r="B36" s="24">
+      <c r="B36" s="21">
         <f t="shared" si="0"/>
         <v>33</v>
       </c>
-      <c r="C36" s="25" t="s">
+      <c r="C36" s="22" t="s">
         <v>31</v>
       </c>
-      <c r="D36" s="26"/>
-      <c r="E36" s="26"/>
-      <c r="F36" s="27"/>
-      <c r="G36" s="31" t="s">
+      <c r="D36" s="23"/>
+      <c r="E36" s="23"/>
+      <c r="F36" s="24"/>
+      <c r="G36" s="27" t="s">
         <v>99</v>
       </c>
-      <c r="H36" s="31"/>
-      <c r="I36" s="31"/>
-      <c r="J36" s="31"/>
-      <c r="K36" s="31" t="s">
+      <c r="H36" s="27"/>
+      <c r="I36" s="27"/>
+      <c r="J36" s="27"/>
+      <c r="K36" s="27" t="s">
         <v>100</v>
       </c>
     </row>
     <row r="37" spans="2:11" x14ac:dyDescent="0.2">
-      <c r="B37" s="18">
+      <c r="B37" s="15">
         <f t="shared" si="0"/>
         <v>34</v>
       </c>
-      <c r="C37" s="21" t="s">
+      <c r="C37" s="18" t="s">
         <v>32</v>
       </c>
-      <c r="D37" s="22"/>
-      <c r="E37" s="22" t="s">
+      <c r="D37" s="19"/>
+      <c r="E37" s="19" t="s">
         <v>58</v>
       </c>
-      <c r="F37" s="23" t="s">
+      <c r="F37" s="20" t="s">
         <v>93</v>
       </c>
-      <c r="G37" s="66" t="s">
-        <v>104</v>
-      </c>
-      <c r="H37" s="66" t="s">
-        <v>104</v>
-      </c>
-      <c r="I37" s="66" t="s">
-        <v>104</v>
-      </c>
-      <c r="J37" s="66" t="s">
-        <v>104</v>
-      </c>
-      <c r="K37" s="66" t="s">
+      <c r="G37" s="62" t="s">
+        <v>104</v>
+      </c>
+      <c r="H37" s="62" t="s">
+        <v>104</v>
+      </c>
+      <c r="I37" s="62" t="s">
+        <v>104</v>
+      </c>
+      <c r="J37" s="62" t="s">
+        <v>104</v>
+      </c>
+      <c r="K37" s="62" t="s">
         <v>104</v>
       </c>
     </row>
     <row r="38" spans="2:11" x14ac:dyDescent="0.2">
-      <c r="B38" s="20">
+      <c r="B38" s="17">
         <f t="shared" si="0"/>
         <v>35</v>
       </c>
-      <c r="C38" s="21" t="s">
+      <c r="C38" s="18" t="s">
         <v>33</v>
       </c>
-      <c r="D38" s="22"/>
-      <c r="E38" s="22"/>
-      <c r="F38" s="23"/>
-      <c r="G38" s="36"/>
-      <c r="H38" s="36"/>
-      <c r="I38" s="36"/>
-      <c r="J38" s="36"/>
-      <c r="K38" s="36"/>
+      <c r="D38" s="19"/>
+      <c r="E38" s="19"/>
+      <c r="F38" s="20"/>
+      <c r="G38" s="32"/>
+      <c r="H38" s="32"/>
+      <c r="I38" s="32"/>
+      <c r="J38" s="32"/>
+      <c r="K38" s="32"/>
     </row>
     <row r="39" spans="2:11" x14ac:dyDescent="0.2">
-      <c r="B39" s="59">
+      <c r="B39" s="55">
         <f t="shared" si="0"/>
         <v>36</v>
       </c>
-      <c r="C39" s="60" t="s">
+      <c r="C39" s="56" t="s">
         <v>34</v>
       </c>
-      <c r="D39" s="47"/>
-      <c r="E39" s="47"/>
-      <c r="F39" s="48"/>
-      <c r="G39" s="49" t="s">
+      <c r="D39" s="43"/>
+      <c r="E39" s="43"/>
+      <c r="F39" s="44"/>
+      <c r="G39" s="45" t="s">
         <v>102</v>
       </c>
-      <c r="H39" s="49"/>
-      <c r="I39" s="49"/>
-      <c r="J39" s="49"/>
-      <c r="K39" s="49"/>
+      <c r="H39" s="45"/>
+      <c r="I39" s="45"/>
+      <c r="J39" s="45" t="s">
+        <v>102</v>
+      </c>
+      <c r="K39" s="45" t="s">
+        <v>102</v>
+      </c>
     </row>
     <row r="40" spans="2:11" x14ac:dyDescent="0.2">
-      <c r="B40" s="20">
+      <c r="B40" s="17">
         <f t="shared" si="0"/>
         <v>37</v>
       </c>
-      <c r="C40" s="21" t="s">
+      <c r="C40" s="18" t="s">
         <v>35</v>
       </c>
-      <c r="D40" s="22"/>
-      <c r="E40" s="22"/>
-      <c r="F40" s="23"/>
-      <c r="G40" s="35" t="s">
+      <c r="D40" s="19"/>
+      <c r="E40" s="19"/>
+      <c r="F40" s="20"/>
+      <c r="G40" s="31" t="s">
         <v>101</v>
       </c>
-      <c r="H40" s="35"/>
-      <c r="I40" s="35"/>
-      <c r="J40" s="35"/>
-      <c r="K40" s="35"/>
+      <c r="H40" s="31"/>
+      <c r="I40" s="31"/>
+      <c r="J40" s="31"/>
+      <c r="K40" s="31"/>
     </row>
     <row r="41" spans="2:11" x14ac:dyDescent="0.2">
-      <c r="B41" s="8">
+      <c r="B41" s="5">
         <f t="shared" si="0"/>
         <v>38</v>
       </c>
-      <c r="C41" s="9" t="s">
+      <c r="C41" s="6" t="s">
         <v>6</v>
       </c>
-      <c r="D41" s="10"/>
-      <c r="E41" s="10"/>
-      <c r="F41" s="11"/>
-      <c r="G41" s="37"/>
-      <c r="H41" s="37"/>
-      <c r="I41" s="37"/>
-      <c r="J41" s="37"/>
-      <c r="K41" s="37"/>
+      <c r="D41" s="7"/>
+      <c r="E41" s="7"/>
+      <c r="F41" s="8"/>
+      <c r="G41" s="33"/>
+      <c r="H41" s="33"/>
+      <c r="I41" s="33"/>
+      <c r="J41" s="33"/>
+      <c r="K41" s="33"/>
     </row>
     <row r="42" spans="2:11" x14ac:dyDescent="0.2">
-      <c r="B42" s="45">
+      <c r="B42" s="41">
         <f t="shared" si="0"/>
         <v>39</v>
       </c>
-      <c r="C42" s="46" t="s">
+      <c r="C42" s="42" t="s">
         <v>36</v>
       </c>
-      <c r="D42" s="47"/>
-      <c r="E42" s="47"/>
-      <c r="F42" s="48"/>
-      <c r="G42" s="55" t="s">
+      <c r="D42" s="43"/>
+      <c r="E42" s="43"/>
+      <c r="F42" s="44"/>
+      <c r="G42" s="51" t="s">
         <v>36</v>
       </c>
-      <c r="H42" s="55"/>
-      <c r="I42" s="55"/>
-      <c r="J42" s="55"/>
-      <c r="K42" s="49"/>
+      <c r="H42" s="51"/>
+      <c r="I42" s="51"/>
+      <c r="J42" s="51"/>
+      <c r="K42" s="45"/>
     </row>
     <row r="43" spans="2:11" ht="16" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="B43" s="50">
+      <c r="B43" s="46">
         <f t="shared" si="0"/>
         <v>40</v>
       </c>
-      <c r="C43" s="51" t="s">
+      <c r="C43" s="47" t="s">
         <v>37</v>
       </c>
-      <c r="D43" s="52"/>
-      <c r="E43" s="52"/>
-      <c r="F43" s="53"/>
-      <c r="G43" s="56" t="s">
+      <c r="D43" s="48"/>
+      <c r="E43" s="48"/>
+      <c r="F43" s="49"/>
+      <c r="G43" s="52" t="s">
         <v>103</v>
       </c>
-      <c r="H43" s="56"/>
-      <c r="I43" s="56"/>
-      <c r="J43" s="56"/>
-      <c r="K43" s="54"/>
+      <c r="H43" s="52"/>
+      <c r="I43" s="52"/>
+      <c r="J43" s="52"/>
+      <c r="K43" s="50"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -2257,7 +2241,7 @@
         <f>0</f>
         <v>0</v>
       </c>
-      <c r="F2" s="57">
+      <c r="F2" s="53">
         <f>E2*6.25</f>
         <v>0</v>
       </c>
@@ -2267,7 +2251,7 @@
         <f>E2+1</f>
         <v>1</v>
       </c>
-      <c r="F3" s="57">
+      <c r="F3" s="53">
         <f t="shared" ref="F3:F9" si="0">E3*6.25</f>
         <v>6.25</v>
       </c>
@@ -2277,7 +2261,7 @@
         <f t="shared" ref="E4:E9" si="1">E3+1</f>
         <v>2</v>
       </c>
-      <c r="F4" s="57">
+      <c r="F4" s="53">
         <f t="shared" si="0"/>
         <v>12.5</v>
       </c>
@@ -2287,7 +2271,7 @@
         <f t="shared" si="1"/>
         <v>3</v>
       </c>
-      <c r="F5" s="57">
+      <c r="F5" s="53">
         <f t="shared" si="0"/>
         <v>18.75</v>
       </c>
@@ -2297,7 +2281,7 @@
         <f t="shared" si="1"/>
         <v>4</v>
       </c>
-      <c r="F6" s="57">
+      <c r="F6" s="53">
         <f t="shared" si="0"/>
         <v>25</v>
       </c>
@@ -2307,7 +2291,7 @@
         <f t="shared" si="1"/>
         <v>5</v>
       </c>
-      <c r="F7" s="57">
+      <c r="F7" s="53">
         <f t="shared" si="0"/>
         <v>31.25</v>
       </c>
@@ -2317,7 +2301,7 @@
         <f t="shared" si="1"/>
         <v>6</v>
       </c>
-      <c r="F8" s="57">
+      <c r="F8" s="53">
         <f t="shared" si="0"/>
         <v>37.5</v>
       </c>
@@ -2327,7 +2311,7 @@
         <f t="shared" si="1"/>
         <v>7</v>
       </c>
-      <c r="F9" s="57">
+      <c r="F9" s="53">
         <f t="shared" si="0"/>
         <v>43.75</v>
       </c>

</xml_diff>